<commit_message>
CTX_BS: Tipo Unita' Resp=UOC + omologazione codici 2026_STG_ + etch 2026 + is_posted=Y freeze 2025 (fonte: SETUP/config/template/fasce/verifiche; prod: PROD_FIX_CTX_BS)
</commit_message>
<xml_diff>
--- a/script/templates/WeRootInterface_BS.xlsx
+++ b/script/templates/WeRootInterface_BS.xlsx
@@ -450,7 +450,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026_OB_PF_STG_BAA9003</t>
+          <t>2026_STG_BAA9003</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026_OB_PF_STG_BSA9090</t>
+          <t>2026_STG_BSA9090</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -504,7 +504,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026_OB_PF_STG_BSTA4800</t>
+          <t>2026_STG_BSTA4800</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9001</t>
+          <t>2026_STG_BAA9001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -558,7 +558,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9902</t>
+          <t>2026_STG_BAA9902</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9903</t>
+          <t>2026_STG_BAA9903</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9904</t>
+          <t>2026_STG_BAA9904</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9905</t>
+          <t>2026_STG_BAA9905</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9906</t>
+          <t>2026_STG_BAA9906</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9907</t>
+          <t>2026_STG_BAA9907</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9908</t>
+          <t>2026_STG_BAA9908</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9909</t>
+          <t>2026_STG_BAA9909</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -774,7 +774,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9910</t>
+          <t>2026_STG_BAA9910</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9911</t>
+          <t>2026_STG_BAA9911</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -828,7 +828,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9912</t>
+          <t>2026_STG_BAA9912</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -855,7 +855,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP0208</t>
+          <t>2026_STG_BSCP0208</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP1404</t>
+          <t>2026_STG_BSCP1404</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP1407</t>
+          <t>2026_STG_BSCP1407</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -936,7 +936,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP1500</t>
+          <t>2026_STG_BSCP1500</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -963,7 +963,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP1800</t>
+          <t>2026_STG_BSCP1800</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -990,7 +990,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP1810</t>
+          <t>2026_STG_BSCP1810</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1017,7 +1017,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP2400</t>
+          <t>2026_STG_BSCP2400</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1044,7 +1044,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCP3500</t>
+          <t>2026_STG_BSCP3500</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1071,7 +1071,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS0510</t>
+          <t>2026_STG_BSCS0510</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS0600</t>
+          <t>2026_STG_BSCS0600</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1125,7 +1125,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS0710</t>
+          <t>2026_STG_BSCS0710</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1152,7 +1152,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS0903</t>
+          <t>2026_STG_BSCS0903</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1179,7 +1179,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1010</t>
+          <t>2026_STG_BSCS1010</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1206,7 +1206,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1402</t>
+          <t>2026_STG_BSCS1402</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1233,7 +1233,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1403</t>
+          <t>2026_STG_BSCS1403</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1260,7 +1260,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1404</t>
+          <t>2026_STG_BSCS1404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1405</t>
+          <t>2026_STG_BSCS1405</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS1600</t>
+          <t>2026_STG_BSCS1600</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1341,7 +1341,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS2230</t>
+          <t>2026_STG_BSCS2230</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSCS3400</t>
+          <t>2026_STG_BSCS3400</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA0120</t>
+          <t>2026_STG_BSEA0120</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1422,7 +1422,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA1000</t>
+          <t>2026_STG_BSEA1000</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1449,7 +1449,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA14081</t>
+          <t>2026_STG_BSEA14081</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1476,7 +1476,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA1410</t>
+          <t>2026_STG_BSEA1410</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1503,7 +1503,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2200</t>
+          <t>2026_STG_BSEA2200</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1530,7 +1530,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2202</t>
+          <t>2026_STG_BSEA2202</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1557,7 +1557,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2210</t>
+          <t>2026_STG_BSEA2210</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1584,7 +1584,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2280</t>
+          <t>2026_STG_BSEA2280</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2500</t>
+          <t>2026_STG_BSEA2500</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1638,7 +1638,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2600</t>
+          <t>2026_STG_BSEA2600</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1665,7 +1665,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA2810</t>
+          <t>2026_STG_BSEA2810</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1692,7 +1692,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSEA4820</t>
+          <t>2026_STG_BSEA4820</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1719,7 +1719,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP0300</t>
+          <t>2026_STG_BSMP0300</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1100</t>
+          <t>2026_STG_BSMP1100</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1773,7 +1773,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1200</t>
+          <t>2026_STG_BSMP1200</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1300</t>
+          <t>2026_STG_BSMP1300</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1827,7 +1827,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1310</t>
+          <t>2026_STG_BSMP1310</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1854,7 +1854,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1320</t>
+          <t>2026_STG_BSMP1320</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP1401</t>
+          <t>2026_STG_BSMP1401</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1908,7 +1908,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP2000</t>
+          <t>2026_STG_BSMP2000</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP2610</t>
+          <t>2026_STG_BSMP2610</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1962,7 +1962,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP3000</t>
+          <t>2026_STG_BSMP3000</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1989,7 +1989,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP3020</t>
+          <t>2026_STG_BSMP3020</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2016,7 +2016,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSMP3700</t>
+          <t>2026_STG_BSMP3700</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2043,7 +2043,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP1900</t>
+          <t>2026_STG_BSOP1900</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP1901</t>
+          <t>2026_STG_BSOP1901</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2097,7 +2097,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP1911</t>
+          <t>2026_STG_BSOP1911</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP2214</t>
+          <t>2026_STG_BSOP2214</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2151,7 +2151,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP3100</t>
+          <t>2026_STG_BSOP3100</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2178,7 +2178,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP3310</t>
+          <t>2026_STG_BSOP3310</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2205,7 +2205,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP3600</t>
+          <t>2026_STG_BSOP3600</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2232,7 +2232,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP3800</t>
+          <t>2026_STG_BSOP3800</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2259,7 +2259,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSOP4000</t>
+          <t>2026_STG_BSOP4000</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2286,7 +2286,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA1002</t>
+          <t>2026_STG_BSTA1002</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2313,7 +2313,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA1003</t>
+          <t>2026_STG_BSTA1003</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2340,7 +2340,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4010</t>
+          <t>2026_STG_BSTA4010</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4100</t>
+          <t>2026_STG_BSTA4100</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2394,7 +2394,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4110</t>
+          <t>2026_STG_BSTA4110</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4111</t>
+          <t>2026_STG_BSTA4111</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2448,7 +2448,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4330</t>
+          <t>2026_STG_BSTA4330</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4600</t>
+          <t>2026_STG_BSTA4600</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2502,7 +2502,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA4810</t>
+          <t>2026_STG_BSTA4810</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2529,7 +2529,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTA5000</t>
+          <t>2026_STG_BSTA5000</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTR0811</t>
+          <t>2026_STG_BSTR0811</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTR0902</t>
+          <t>2026_STG_BSTR0902</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2610,7 +2610,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTR2010</t>
+          <t>2026_STG_BSTR2010</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSTR2213</t>
+          <t>2026_STG_BSTR2213</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2664,7 +2664,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU1405</t>
+          <t>2026_STG_BSU1405</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2691,7 +2691,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU1409</t>
+          <t>2026_STG_BSU1409</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2718,7 +2718,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU4500</t>
+          <t>2026_STG_BSU4500</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2745,7 +2745,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU4700</t>
+          <t>2026_STG_BSU4700</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2772,7 +2772,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU7200</t>
+          <t>2026_STG_BSU7200</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU9095</t>
+          <t>2026_STG_BSU9095</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU9096</t>
+          <t>2026_STG_BSU9096</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2853,7 +2853,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BSU9208</t>
+          <t>2026_STG_BSU9208</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2880,7 +2880,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026_OB_STG_BAA9913</t>
+          <t>2026_STG_BAA9913</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">

</xml_diff>

<commit_message>
CTX_BS: etichette PF_STG_<anno> + titolo 'Scheda' (2026) + hideTreeView CTX_BS/CTX_EP; script prod unico timestampato PROD_FIX_CTX_BS_20260922 (sostituisce PROD_FIX_CTX_BS + CONFIG_FIX); template Nome Scheda + SETUP V001a2 esteso a CTX_EP
</commit_message>
<xml_diff>
--- a/script/templates/WeRootInterface_BS.xlsx
+++ b/script/templates/WeRootInterface_BS.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio ispettivo</t>
+          <t>Scheda Performance Strategica UOC Servizio ispettivo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -482,7 +482,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Direzione sanitaria aziendale</t>
+          <t>Scheda Performance Strategica UOC Direzione sanitaria aziendale</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Farmacia Umaca</t>
+          <t>Scheda Performance Strategica UOC Farmacia Umaca</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Segretariato Generale</t>
+          <t>Scheda Performance Strategica UOC Segretariato Generale</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ufficio Legale e Avvocatura (ULA)</t>
+          <t>Scheda Performance Strategica UOC Ufficio Legale e Avvocatura (ULA)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gestione Risorse Umane</t>
+          <t>Scheda Performance Strategica UOC Gestione Risorse Umane</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Affari Generali</t>
+          <t>Scheda Performance Strategica UOC Affari Generali</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gestione Economica e Finanziaria (GEF)</t>
+          <t>Scheda Performance Strategica UOC Gestione Economica e Finanziaria (GEF)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Provveditorato ed Economato</t>
+          <t>Scheda Performance Strategica UOC Provveditorato ed Economato</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gestione Risorse Tecniche</t>
+          <t>Scheda Performance Strategica UOC Gestione Risorse Tecniche</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Pianificazione e Controllo di Gestione</t>
+          <t>Scheda Performance Strategica UOC Pianificazione e Controllo di Gestione</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gestione Sistemi Informatici (GSI)</t>
+          <t>Scheda Performance Strategica UOC Gestione Sistemi Informatici (GSI)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ingegneria Clinica</t>
+          <t>Scheda Performance Strategica UOC Ingegneria Clinica</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio Protezione, Prevenzione e Sicurezza Antincendio</t>
+          <t>Scheda Performance Strategica UOC Servizio Protezione, Prevenzione e Sicurezza Antincendio</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Comunicazione e Innovazione</t>
+          <t>Scheda Performance Strategica UOC Comunicazione e Innovazione</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ortopedia 2</t>
+          <t>Scheda Performance Strategica UOC Ortopedia 2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Maculopatia e Patologia Vitreo - retinica</t>
+          <t>Scheda Performance Strategica UOC Maculopatia e Patologia Vitreo - retinica</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Andrologia</t>
+          <t>Scheda Performance Strategica UOC Andrologia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Urologia</t>
+          <t>Scheda Performance Strategica UOC Urologia</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Otorinolaringoiatria</t>
+          <t>Scheda Performance Strategica UOC Otorinolaringoiatria</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Oculistica</t>
+          <t>Scheda Performance Strategica UOC Oculistica</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ortopedia 1</t>
+          <t>Scheda Performance Strategica UOC Ortopedia 1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ostetricia e ginecologia</t>
+          <t>Scheda Performance Strategica UOC Ostetricia e ginecologia</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Odontostomatologia</t>
+          <t>Scheda Performance Strategica UOC Odontostomatologia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia generale ad indirizzo oncologico mininvasivo con alta specializzazione esofago-gastrica</t>
+          <t>Scheda Performance Strategica UOC Chirurgia generale ad indirizzo oncologico mininvasivo con alta specializzazione esofago-gastrica</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia generale ad alta specializzazione gastroenterologica</t>
+          <t>Scheda Performance Strategica UOC Chirurgia generale ad alta specializzazione gastroenterologica</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia vascolare ed endovascolare</t>
+          <t>Scheda Performance Strategica UOC Chirurgia vascolare ed endovascolare</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Terapia intensiva post-operatoria</t>
+          <t>Scheda Performance Strategica UOC Terapia intensiva post-operatoria</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia senologica</t>
+          <t>Scheda Performance Strategica UOC Chirurgia senologica</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia metabolica e dei grandi obesi</t>
+          <t>Scheda Performance Strategica UOC Chirurgia metabolica e dei grandi obesi</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Week e Day Surgery</t>
+          <t>Scheda Performance Strategica UOC Week e Day Surgery</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia della Tiroide e Paratiroidi</t>
+          <t>Scheda Performance Strategica UOC Chirurgia della Tiroide e Paratiroidi</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia generale ad alta specializzazione pancreatica</t>
+          <t>Scheda Performance Strategica UOC Chirurgia generale ad alta specializzazione pancreatica</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia maxillo-facciale</t>
+          <t>Scheda Performance Strategica UOC Chirurgia maxillo-facciale</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia toracica</t>
+          <t>Scheda Performance Strategica UOC Chirurgia toracica</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia plastica ricostruttiva</t>
+          <t>Scheda Performance Strategica UOC Chirurgia plastica ricostruttiva</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina DEA e complessita clinica</t>
+          <t>Scheda Performance Strategica UOC Medicina DEA e complessita clinica</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Coordinamento attivita prelievi organi e tessuti</t>
+          <t>Scheda Performance Strategica UOC Coordinamento attivita prelievi organi e tessuti</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Trauma Center</t>
+          <t>Scheda Performance Strategica UOC Trauma Center</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia d urgenza</t>
+          <t>Scheda Performance Strategica UOC Chirurgia d urgenza</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Pronto Soccorso OBI e Medicina di Emergenza e Urgenza</t>
+          <t>Scheda Performance Strategica UOC Pronto Soccorso OBI e Medicina di Emergenza e Urgenza</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Rianimazione DEA</t>
+          <t>Scheda Performance Strategica UOC Rianimazione DEA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Terapia intensiva grandi ustionati</t>
+          <t>Scheda Performance Strategica UOC Terapia intensiva grandi ustionati</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Neurochirurgia</t>
+          <t>Scheda Performance Strategica UOC Neurochirurgia</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Neurologia</t>
+          <t>Scheda Performance Strategica UOC Neurologia</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Terapia intensiva neonatale e neonatologia</t>
+          <t>Scheda Performance Strategica UOC Terapia intensiva neonatale e neonatologia</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Cardiologia con UTIC</t>
+          <t>Scheda Performance Strategica UOC Cardiologia con UTIC</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina interna 3</t>
+          <t>Scheda Performance Strategica UOC Medicina interna 3</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina interna 1</t>
+          <t>Scheda Performance Strategica UOC Medicina interna 1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Endocrinologia</t>
+          <t>Scheda Performance Strategica UOC Endocrinologia</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina interna 2</t>
+          <t>Scheda Performance Strategica UOC Medicina interna 2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Riabilitazione specialistica</t>
+          <t>Scheda Performance Strategica UOC Riabilitazione specialistica</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina a indirizzo geriatrico</t>
+          <t>Scheda Performance Strategica UOC Medicina a indirizzo geriatrico</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Diabetologia</t>
+          <t>Scheda Performance Strategica UOC Diabetologia</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Cardiologia</t>
+          <t>Scheda Performance Strategica UOC Cardiologia</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Neurofisiopatologia</t>
+          <t>Scheda Performance Strategica UOC Neurofisiopatologia</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Dermatologia</t>
+          <t>Scheda Performance Strategica UOC Dermatologia</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Nefrologia con emodialisi in elezione e in emergenza</t>
+          <t>Scheda Performance Strategica UOC Nefrologia con emodialisi in elezione e in emergenza</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Detenuti</t>
+          <t>Scheda Performance Strategica UOC Detenuti</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ematologia</t>
+          <t>Scheda Performance Strategica UOC Ematologia</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Malattie rare del globulo rosso</t>
+          <t>Scheda Performance Strategica UOC Malattie rare del globulo rosso</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Ematologia con trapianti di cellule staminali ematopoietiche (CSE) e Terapia Intensiva</t>
+          <t>Scheda Performance Strategica UOC Ematologia con trapianti di cellule staminali ematopoietiche (CSE) e Terapia Intensiva</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio di terapia del dolore</t>
+          <t>Scheda Performance Strategica UOC Servizio di terapia del dolore</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Pneumologia</t>
+          <t>Scheda Performance Strategica UOC Pneumologia</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Oncologia</t>
+          <t>Scheda Performance Strategica UOC Oncologia</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Pneumologia e terapia semintensiva respiratoria</t>
+          <t>Scheda Performance Strategica UOC Pneumologia e terapia semintensiva respiratoria</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio di pneumologia interventistica</t>
+          <t>Scheda Performance Strategica UOC Servizio di pneumologia interventistica</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Fisiopatologie respiratorie</t>
+          <t>Scheda Performance Strategica UOC Fisiopatologie respiratorie</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Fisica sanitaria</t>
+          <t>Scheda Performance Strategica UOC Fisica sanitaria</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Diagnostica senologica</t>
+          <t>Scheda Performance Strategica UOC Diagnostica senologica</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio di immunoematologia e medicina trasfusionale</t>
+          <t>Scheda Performance Strategica UOC Servizio di immunoematologia e medicina trasfusionale</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Neuroradiologia</t>
+          <t>Scheda Performance Strategica UOC Neuroradiologia</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Radiologia generale e di pronto soccorso</t>
+          <t>Scheda Performance Strategica UOC Radiologia generale e di pronto soccorso</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Medicina nucleare</t>
+          <t>Scheda Performance Strategica UOC Medicina nucleare</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Radiologia vascolare ed interventistica</t>
+          <t>Scheda Performance Strategica UOC Radiologia vascolare ed interventistica</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Anatomia patologica</t>
+          <t>Scheda Performance Strategica UOC Anatomia patologica</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Genetica medica e di laboratorio</t>
+          <t>Scheda Performance Strategica UOC Genetica medica e di laboratorio</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Patologia clinica</t>
+          <t>Scheda Performance Strategica UOC Patologia clinica</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Epatologia</t>
+          <t>Scheda Performance Strategica UOC Epatologia</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Chirurgia epatobiliare e trapianto di fegato</t>
+          <t>Scheda Performance Strategica UOC Chirurgia epatobiliare e trapianto di fegato</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gastroenterologia</t>
+          <t>Scheda Performance Strategica UOC Gastroenterologia</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Terapia intensiva fegato</t>
+          <t>Scheda Performance Strategica UOC Terapia intensiva fegato</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Pre-ospedalizzazione centralizzata</t>
+          <t>Scheda Performance Strategica UOC Pre-ospedalizzazione centralizzata</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Gestione servizi di supporto alla direzione sanitaria e dei posti letto</t>
+          <t>Scheda Performance Strategica UOC Gestione servizi di supporto alla direzione sanitaria e dei posti letto</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Risk Management</t>
+          <t>Scheda Performance Strategica UOC Risk Management</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Formazione, ricerca e cooperazione internazionale</t>
+          <t>Scheda Performance Strategica UOC Formazione, ricerca e cooperazione internazionale</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Appropriatezza ed epidemiologia valutativa</t>
+          <t>Scheda Performance Strategica UOC Appropriatezza ed epidemiologia valutativa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Programmazione e pianificazione sanitaria</t>
+          <t>Scheda Performance Strategica UOC Programmazione e pianificazione sanitaria</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Direzione infermieristica tecnica e riabilitativa</t>
+          <t>Scheda Performance Strategica UOC Direzione infermieristica tecnica e riabilitativa</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Attivita in libera professione intramoenia</t>
+          <t>Scheda Performance Strategica UOC Attivita in libera professione intramoenia</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Investimenti e Energy Management</t>
+          <t>Scheda Performance Strategica UOC Investimenti e Energy Management</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">

</xml_diff>